<commit_message>
data: publish 2026-10-10 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-10-182路.xlsx
+++ b/data/export/2026-10-10-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>77分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>4/13</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,17 +812,17 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -820,13 +832,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -854,32 +870,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -887,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,33 +931,37 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -965,32 +989,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>76分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,17 +1050,17 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1042,13 +1070,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>76.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1148,7 +1180,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1159,7 +1191,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1252,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1302,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1363,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1413,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1421,22 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A32298D</t>
+          <t>沪A02126A</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1437,12 +1469,12 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:32</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1456,7 +1488,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1492,7 +1524,903 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:32</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>4/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>2/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-10 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-10-182路.xlsx
+++ b/data/export/2026-10-10-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC31"/>
+  <dimension ref="A1:AC34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,14 +827,14 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
           <t>82.0</t>
@@ -842,7 +842,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA7" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>82.5</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2481,14 +2481,14 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
           <t>82.0</t>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -2639,32 +2639,36 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>88分钟</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2672,7 +2676,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2696,17 +2700,17 @@
       </c>
       <c r="W19" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z19" s="2" t="inlineStr">
@@ -2716,7 +2720,7 @@
       </c>
       <c r="AA19" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB19" s="2" t="inlineStr">
@@ -2726,7 +2730,7 @@
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -2754,32 +2758,36 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
           <t>07:51</t>
@@ -2787,7 +2795,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2811,17 +2819,17 @@
       </c>
       <c r="W20" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z20" s="2" t="inlineStr">
@@ -2831,13 +2839,17 @@
       </c>
       <c r="AA20" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB20" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="inlineStr">
+        <is>
+          <t>83.0</t>
+        </is>
+      </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -2865,32 +2877,36 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>86分钟</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
           <t>06:11</t>
@@ -2898,7 +2914,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2922,37 +2938,37 @@
       </c>
       <c r="W21" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA21" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>82.5</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3029,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3067,7 +3083,7 @@
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3144,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3239,7 +3255,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3293,7 +3309,7 @@
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3370,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3408,7 +3424,7 @@
       </c>
       <c r="AC25" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3485,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3523,7 +3539,7 @@
       </c>
       <c r="AC26" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3600,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3638,7 +3654,7 @@
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3715,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3753,7 +3769,7 @@
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3830,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3868,7 +3884,7 @@
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3945,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -3991,22 +4007,22 @@
       <c r="A31" s="2" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>沪A31073D</t>
+          <t>沪A67983D</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -4044,7 +4060,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4058,47 +4074,392 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr">
         <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>82.0</t>
+        </is>
+      </c>
+      <c r="AC31" s="2" t="inlineStr">
+        <is>
+          <t>2/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
           <t>10:15</t>
         </is>
       </c>
-      <c r="V31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W31" s="2" t="inlineStr">
+      <c r="W32" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X31" s="2" t="inlineStr">
-        <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="Y31" s="2" t="inlineStr">
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="Z31" s="2" t="inlineStr">
+      <c r="Z32" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA31" s="2" t="inlineStr">
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr">
+        <is>
+          <t>88.0</t>
+        </is>
+      </c>
+      <c r="AC32" s="2" t="inlineStr">
+        <is>
+          <t>8/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB31" s="2" t="inlineStr">
-        <is>
-          <t>88.0</t>
-        </is>
-      </c>
-      <c r="AC31" s="2" t="inlineStr">
-        <is>
-          <t>7/14</t>
+      <c r="AB33" s="2" t="inlineStr">
+        <is>
+          <t>89.0</t>
+        </is>
+      </c>
+      <c r="AC33" s="2" t="inlineStr">
+        <is>
+          <t>9/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB34" s="2" t="inlineStr">
+        <is>
+          <t>82.5</t>
+        </is>
+      </c>
+      <c r="AC34" s="2" t="inlineStr">
+        <is>
+          <t>3/14</t>
         </is>
       </c>
     </row>

</xml_diff>